<commit_message>
Add USyd application and update skill/master resume
- New application: Head of Student Insights and Analytics — University of Sydney
  with tailored resume and job ad
- Updated resume-tailor skill: added job requirement importance ranking logic,
  flexibility allowance, LinkedIn URL support, bullet style rules,
  post-tailoring update workflow, and XML namespace fix
- Updated Resume_Master.docx: improved Areas of Expertise with new capability
  phrasings, merged Tech Stack categories, generalized platform names
- Updated Skills_Gap_Analysis.xlsx: added USyd column with 38 skills assessed
</commit_message>
<xml_diff>
--- a/Skills_Gap_Analysis.xlsx
+++ b/Skills_Gap_Analysis.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,17 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00007A33"/>
+    </font>
+    <font>
+      <color rgb="00D4A017"/>
     </font>
   </fonts>
   <fills count="7">
@@ -98,7 +109,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -120,11 +131,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -165,6 +220,13 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -530,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -545,14 +607,24 @@
           <t>Skills &amp; Capabilities Matrix</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="20" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="22" t="inlineStr">
+        <is>
+          <t>USyd - Head of Student Insights &amp; Analytics</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 29 May 2026</t>
+          <t>Last updated: 30 May 2026</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>30 May 2026</t>
         </is>
       </c>
     </row>
@@ -599,6 +671,11 @@
           <t>Defined &amp; executed analytics strategy for Group Treasury</t>
         </is>
       </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -621,6 +698,11 @@
           <t>30+ Power BI dashboards, Tableau</t>
         </is>
       </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -643,6 +725,11 @@
           <t>Predictive modelling project; attribution in sticky factors work</t>
         </is>
       </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -665,6 +752,11 @@
           <t>$5B deposit release via segmentation analysis</t>
         </is>
       </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -687,6 +779,11 @@
           <t>Daily balance sheet modelling on large datasets</t>
         </is>
       </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -709,6 +806,11 @@
           <t>Daily-execution predictive model for funding analysis</t>
         </is>
       </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -731,6 +833,11 @@
           <t>Designed reporting frameworks for Group Treasury</t>
         </is>
       </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -753,6 +860,11 @@
           <t>$5B unlocked, $120M annual savings</t>
         </is>
       </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -775,6 +887,11 @@
           <t>Presented to exec stakeholders; translated complex findings</t>
         </is>
       </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -797,6 +914,11 @@
           <t>Designed data solutions using Dataiku, CDH, Alteryx</t>
         </is>
       </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -819,6 +941,11 @@
           <t>200+ licensees adopted; 30+ dashboards delivered</t>
         </is>
       </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -841,6 +968,11 @@
           <t>Grew analytics community from 30 to 200+ practitioners</t>
         </is>
       </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -863,6 +995,11 @@
           <t>Led teams of 10+ across Treasury, Risk, COG, Business</t>
         </is>
       </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -885,6 +1022,11 @@
           <t>Transformed finance team into analytics function in 12 months</t>
         </is>
       </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -907,6 +1049,11 @@
           <t>200+ hours training; 150+ certifications; 500+ attendees</t>
         </is>
       </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -929,6 +1076,11 @@
           <t>Evolved operating model for data &amp; analytics at Group Treasury</t>
         </is>
       </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1326,6 +1478,8 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
@@ -1378,6 +1532,109 @@
       <c r="B45" s="12" t="inlineStr">
         <is>
           <t>Gap — no direct experience; transferable skills may apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Data &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Market Research &amp; Trend Analysis</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="E46" s="24" t="inlineStr">
+        <is>
+          <t>Predictive modelling &amp; trend analysis for commercial decisions; adjacent domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Data &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Institutional Reporting Modernisation</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="E47" s="23" t="inlineStr">
+        <is>
+          <t>Enterprise-wide Power BI &amp; Alteryx adoption; 200+ certified users; 30+ dashboards</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Stakeholder</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Influencing Diverse Audiences incl. Executives</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="E48" s="23" t="inlineStr">
+        <is>
+          <t>Trusted advisor to senior leadership; AI Forum founder; cross-functional stakeholder mgmt</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Leadership &amp; Team</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Talent &amp; Capability Uplift</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="E49" s="23" t="inlineStr">
+        <is>
+          <t>200+ hrs training; learning pathways adopted Macquarie-wide; 200+ certifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Summary for USyd - Head of Student Insights &amp; Analytics:</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Strong matches: 31 (82%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Present / Understated: 7 (18%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Gaps: 0 (0%)</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1415,14 +1672,14 @@
           <t>Gap Analysis &amp; Development Priorities</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="20" t="n"/>
+      <c r="D1" s="21" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Last updated: 29 May 2026</t>
+          <t>Last updated: 30 May 2026</t>
         </is>
       </c>
     </row>
@@ -1610,6 +1867,72 @@
       <c r="B16" s="19" t="inlineStr">
         <is>
           <t>3 (9%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Higher education / tertiary sector experience (advantageous not required)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>USyd — Head of Student Insights &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Leverage USyd Master of Data Science alumni status (2021). Frame FS analytics leadership as industry-agnostic; highlight focus on measurable outcomes applicable to university context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Direct student insights / student experience intelligence experience</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>USyd — Head of Student Insights &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Reframe customer segmentation &amp; insights work through student analytics lens. Commercial customer analytics skills directly transferable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Traditional market research background</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>USyd — Head of Student Insights &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Predictive modelling, trend analysis and commercial insight generation are functionally equivalent. Position analytics-led research as a modern alternative to traditional market research methods.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add QBE Insurance application and update source of truth files
- QBE resume tailored for Data & AI Strategy and Value Assurance, Senior Manager role
- Job ad saved as .docx in application folder
- Resume_Master.docx: added 8 new AoE phrasings, merged Data Viz into Analytics & Data Platforms
- Skills_Gap_Analysis.xlsx: added QBE column (68% strong match), 3 new gaps identified
</commit_message>
<xml_diff>
--- a/Skills_Gap_Analysis.xlsx
+++ b/Skills_Gap_Analysis.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,6 +69,13 @@
     </font>
     <font>
       <color rgb="00D4A017"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="7">
@@ -179,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -227,6 +234,11 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -592,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -615,6 +627,11 @@
           <t>USyd - Head of Student Insights &amp; Analytics</t>
         </is>
       </c>
+      <c r="F1" s="25" t="inlineStr">
+        <is>
+          <t>QBE - Data &amp; AI Strategy and Value Assurance</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -627,7 +644,13 @@
           <t>30 May 2026</t>
         </is>
       </c>
-    </row>
+      <c r="F2" s="26" t="inlineStr">
+        <is>
+          <t>30 May 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -649,6 +672,11 @@
           <t>Evidence / Notes</t>
         </is>
       </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>QBE - Data &amp; AI Strategy and Value Assurance</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -676,6 +704,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -703,6 +736,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F6" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -730,6 +768,11 @@
           <t>○</t>
         </is>
       </c>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -757,6 +800,11 @@
           <t>○</t>
         </is>
       </c>
+      <c r="F8" s="27" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -784,6 +832,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -811,6 +864,11 @@
           <t>○</t>
         </is>
       </c>
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>△</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -838,6 +896,11 @@
           <t>○</t>
         </is>
       </c>
+      <c r="F11" s="27" t="inlineStr">
+        <is>
+          <t>△</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -865,6 +928,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F12" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -892,6 +960,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F13" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -919,6 +992,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F14" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -946,6 +1024,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F15" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -973,6 +1056,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F16" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1000,6 +1088,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F17" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1027,6 +1120,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1054,6 +1152,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F19" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1081,6 +1184,11 @@
           <t>✓</t>
         </is>
       </c>
+      <c r="F20" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1103,6 +1211,11 @@
           <t>Founded GT AI Forum; contributed to group-wide AI strategy</t>
         </is>
       </c>
+      <c r="F21" s="27" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1125,6 +1238,11 @@
           <t>Evaluated &amp; onboarded Alteryx, Power BI; explored Gen AI</t>
         </is>
       </c>
+      <c r="F22" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1147,6 +1265,11 @@
           <t>Developed AI agents; connected with COG AI teams</t>
         </is>
       </c>
+      <c r="F23" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1169,6 +1292,11 @@
           <t>Trusted advisor to exec on data strategy &amp; investments</t>
         </is>
       </c>
+      <c r="F24" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1191,6 +1319,11 @@
           <t>Partnered across business, risk, finance, technology</t>
         </is>
       </c>
+      <c r="F25" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1213,6 +1346,11 @@
           <t>Macquarie, CBA, Charter Hall — all matrix environments</t>
         </is>
       </c>
+      <c r="F26" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1235,6 +1373,11 @@
           <t>Articulated technical findings to non-technical stakeholders</t>
         </is>
       </c>
+      <c r="F27" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1257,6 +1400,11 @@
           <t>Worked with data leaders across GT, COG, FPE</t>
         </is>
       </c>
+      <c r="F28" s="27" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1279,6 +1427,11 @@
           <t>Daily use for data analysis and solution design</t>
         </is>
       </c>
+      <c r="F29" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1301,6 +1454,11 @@
           <t>Co-led Alteryx onboarding; led Dataiku-based solutions</t>
         </is>
       </c>
+      <c r="F30" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1323,6 +1481,11 @@
           <t>Enterprise dashboards; user enablement</t>
         </is>
       </c>
+      <c r="F31" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1345,6 +1508,11 @@
           <t>AI agents; AI Forum; personal proficiency</t>
         </is>
       </c>
+      <c r="F32" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1367,6 +1535,11 @@
           <t>Delivered 10+ projects in Agile environments</t>
         </is>
       </c>
+      <c r="F33" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1389,6 +1562,11 @@
           <t>UDA governance; model risk; APRA CPG 235; 3LoD</t>
         </is>
       </c>
+      <c r="F34" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -1411,6 +1589,11 @@
           <t>Built independent data solution review function</t>
         </is>
       </c>
+      <c r="F35" s="27" t="inlineStr">
+        <is>
+          <t>△</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1433,6 +1616,11 @@
           <t>Career entirely in financial services — transferable analytics skills</t>
         </is>
       </c>
+      <c r="F36" s="27" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -1455,6 +1643,11 @@
           <t>B2B financial services; limited B2C/customer-experience framing</t>
         </is>
       </c>
+      <c r="F37" s="27" t="inlineStr">
+        <is>
+          <t>△</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -1475,164 +1668,318 @@
       <c r="D38" s="7" t="inlineStr">
         <is>
           <t>Australia-focused roles; APAC not explicit</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="inlineStr">
+        <is>
+          <t>△</t>
         </is>
       </c>
     </row>
     <row r="39"/>
     <row r="40"/>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="A41" s="26" t="inlineStr">
+        <is>
+          <t>Industry / Context</t>
+        </is>
+      </c>
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>Insurance Sector Experience</t>
+        </is>
+      </c>
+      <c r="D41" s="26" t="inlineStr">
+        <is>
+          <t>Career entirely in banking/FS. QBE is APRA-regulated so governance transfers. Insurance domain (brokers, underwriters) not present.</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="26" t="inlineStr">
+        <is>
+          <t>Strategy &amp; Thought Leadership</t>
+        </is>
+      </c>
+      <c r="B42" s="26" t="inlineStr">
+        <is>
+          <t>Value Realisation &amp; Benefits Tracking</t>
+        </is>
+      </c>
+      <c r="D42" s="26" t="inlineStr">
+        <is>
+          <t>$5B assets unlocked; $120M annual savings; 80,000+ FTE hours saved — documented value delivery</t>
+        </is>
+      </c>
+      <c r="F42" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="26" t="inlineStr">
+        <is>
+          <t>Strategy &amp; Thought Leadership</t>
+        </is>
+      </c>
+      <c r="B43" s="26" t="inlineStr">
+        <is>
+          <t>Business Case Development</t>
+        </is>
+      </c>
+      <c r="D43" s="26" t="inlineStr">
+        <is>
+          <t>Built business cases for data &amp; AI initiatives at Macquarie, articulating benefits, costs, strategic value</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="26" t="inlineStr">
+        <is>
+          <t>Strategy &amp; Thought Leadership</t>
+        </is>
+      </c>
+      <c r="B44" s="26" t="inlineStr">
+        <is>
+          <t>Enterprise Strategy Development &amp; Refresh</t>
+        </is>
+      </c>
+      <c r="D44" s="26" t="inlineStr">
+        <is>
+          <t>Defined and executed end-to-end data &amp; analytics strategy for Group Treasury</t>
+        </is>
+      </c>
+      <c r="F44" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t>Strategy &amp; Thought Leadership</t>
+        </is>
+      </c>
+      <c r="B45" s="26" t="inlineStr">
+        <is>
+          <t>Portfolio Governance &amp; Value Assurance</t>
+        </is>
+      </c>
+      <c r="D45" s="26" t="inlineStr">
+        <is>
+          <t>Independent review function + SDLC governance; portfolio-level assurance not explicit</t>
+        </is>
+      </c>
+      <c r="F45" s="27" t="inlineStr">
+        <is>
+          <t>△</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="26" t="inlineStr">
+        <is>
+          <t>Stakeholder &amp; Communication</t>
+        </is>
+      </c>
+      <c r="B46" s="26" t="inlineStr">
+        <is>
+          <t>Board &amp; Senior Leadership Reporting</t>
+        </is>
+      </c>
+      <c r="D46" s="26" t="inlineStr">
+        <is>
+          <t>Prepared materials for executive forums; ensured visibility at senior leadership levels</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t>Stakeholder &amp; Communication</t>
+        </is>
+      </c>
+      <c r="B47" s="26" t="inlineStr">
+        <is>
+          <t>OKR Development &amp; Alignment</t>
+        </is>
+      </c>
+      <c r="D47" s="26" t="inlineStr">
+        <is>
+          <t>Strategic planning and KPI framework experience; OKR-specific terminology not in resume</t>
+        </is>
+      </c>
+      <c r="F47" s="27" t="inlineStr">
+        <is>
+          <t>△</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">  ✓</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>Strong — direct, demonstrable experience</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="13" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  ○</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>Present — experience exists but not prominent</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="13" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  △</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>Understated — capability exists but needs reframing</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="14" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  ✗</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B52" s="12" t="inlineStr">
         <is>
           <t>Gap — no direct experience; transferable skills may apply</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Data &amp; Analytics</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Market Research &amp; Trend Analysis</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="E46" s="24" t="inlineStr">
-        <is>
-          <t>Predictive modelling &amp; trend analysis for commercial decisions; adjacent domain</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Data &amp; Analytics</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Institutional Reporting Modernisation</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="E47" s="23" t="inlineStr">
-        <is>
-          <t>Enterprise-wide Power BI &amp; Alteryx adoption; 200+ certified users; 30+ dashboards</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Stakeholder</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Influencing Diverse Audiences incl. Executives</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="E48" s="23" t="inlineStr">
-        <is>
-          <t>Trusted advisor to senior leadership; AI Forum founder; cross-functional stakeholder mgmt</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Leadership &amp; Team</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Talent &amp; Capability Uplift</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="E49" s="23" t="inlineStr">
-        <is>
-          <t>200+ hrs training; learning pathways adopted Macquarie-wide; 200+ certifications</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Summary for USyd - Head of Student Insights &amp; Analytics:</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Strong matches: 31 (82%)</t>
+          <t>Data &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Market Research &amp; Trend Analysis</t>
+        </is>
+      </c>
+      <c r="E53" s="24" t="inlineStr">
+        <is>
+          <t>Predictive modelling &amp; trend analysis for commercial decisions; adjacent domain</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Present / Understated: 7 (18%)</t>
+          <t>Data &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Institutional Reporting Modernisation</t>
+        </is>
+      </c>
+      <c r="E54" s="23" t="inlineStr">
+        <is>
+          <t>Enterprise-wide Power BI &amp; Alteryx adoption; 200+ certified users; 30+ dashboards</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
+        <is>
+          <t>Stakeholder</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Influencing Diverse Audiences incl. Executives</t>
+        </is>
+      </c>
+      <c r="E55" s="23" t="inlineStr">
+        <is>
+          <t>Trusted advisor to senior leadership; AI Forum founder; cross-functional stakeholder mgmt</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Leadership &amp; Team</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Talent &amp; Capability Uplift</t>
+        </is>
+      </c>
+      <c r="E56" s="23" t="inlineStr">
+        <is>
+          <t>200+ hrs training; learning pathways adopted Macquarie-wide; 200+ certifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Summary for USyd - Head of Student Insights &amp; Analytics:</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Strong matches: 31 (82%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Present / Understated: 7 (18%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t>Gaps: 0 (0%)</t>
         </is>
@@ -1657,7 +2004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1683,6 +2030,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -1815,122 +2163,190 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>Insurance sector experience</t>
+        </is>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Medium-High</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="inlineStr">
+        <is>
+          <t>QBE - Data &amp; AI Strategy and Value Assurance</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Primary gap. No insurance sector experience. Mitigation: QBE is APRA-regulated — data governance (CPG 235, 3LoD) transfers directly. Emphasise transferable analytics leadership and FS regulatory depth. Research QBE products and broker/underwriter ecosystem before interview.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>Portfolio value assurance / investment assurance</t>
+        </is>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Low-Medium</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>QBE - Data &amp; AI Strategy and Value Assurance</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>Independent review function and SDLC governance at Macquarie provide adjacent experience. Business case development and value tracking ($5B, $120M) demonstrate value mindset. Gap is in formal portfolio-level assurance frameworks — frame existing governance work as foundational.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>OKR development &amp; alignment experience</t>
+        </is>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>QBE - Data &amp; AI Strategy and Value Assurance</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>OKR terminology not in resume. Strategic planning, KPI framework design, and operating model work are functionally equivalent. Bridge by framing existing strategic planning work through OKR lens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Summary:</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Total skills assessed:</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Strong matches:</t>
-        </is>
-      </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>19 (58%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Present / Understated:</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>11 (33%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
+          <t>Total skills assessed:</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Strong matches:</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>19 (58%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Present / Understated:</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>11 (33%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
           <t>Gaps:</t>
         </is>
       </c>
-      <c r="B16" s="19" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>3 (9%)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Higher education / tertiary sector experience (advantageous not required)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>USyd — Head of Student Insights &amp; Analytics</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Leverage USyd Master of Data Science alumni status (2021). Frame FS analytics leadership as industry-agnostic; highlight focus on measurable outcomes applicable to university context.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Direct student insights / student experience intelligence experience</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Low-Medium</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>USyd — Head of Student Insights &amp; Analytics</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Reframe customer segmentation &amp; insights work through student analytics lens. Commercial customer analytics skills directly transferable.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Traditional market research background</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>USyd — Head of Student Insights &amp; Analytics</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Predictive modelling, trend analysis and commercial insight generation are functionally equivalent. Position analytics-led research as a modern alternative to traditional market research methods.</t>
         </is>

</xml_diff>